<commit_message>
chore: add Stage 1 WPL evidence and simulated assurance
</commit_message>
<xml_diff>
--- a/evidence/source_register.xlsx
+++ b/evidence/source_register.xlsx
@@ -135,12 +135,12 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>sources/bristol-council/webpages/bcc_workplace_parking_levy_project_page.html</t>
+          <t>evidence/raw/bristol-city-council/src-bcc-0001_bcc-workplace-parking-levy-project-page.html</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>seeded_not_downloaded</t>
+          <t>downloaded</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -150,12 +150,12 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t/>
+          <t>697d485ea02ee03484db03a9fd8023be2706dcc3467264e400acd93717b8e84f</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -212,12 +212,12 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>sources/bristol-council/webpages/bcc_news_further_information_bristol_wpl_2026-02-23.html</t>
+          <t>evidence/raw/bristol-city-council/src-bcc-0002_bcc-news-further-information-bristol-wpl-2026-02-23.html</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>seeded_not_downloaded</t>
+          <t>downloaded</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -227,12 +227,12 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t/>
+          <t>f4f3be4ca5e6a08c0789cd6108dbbb415d7ef203c3469073a1334a8dd97088f6</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
@@ -289,12 +289,12 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>sources/bristol-council/committee-reports/2024-09-12/committee_report_workplace_parking_levy_2024-09-12.pdf</t>
+          <t>evidence/raw/bristol-city-council/src-bcc-0003_committee-report-workplace-parking-levy-2024-09-12.pdf</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>seeded_not_downloaded</t>
+          <t>downloaded</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -304,12 +304,12 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t/>
+          <t>6c15764ee31f3e495dd3b168be34a50e676c5f203b7b87ceebfbafc1a9c8fff6</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -366,12 +366,12 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>sources/bristol-council/committee-reports/2024-09-12/decision_notice_transport_connectivity_policy_committee_2024-09-12.pdf</t>
+          <t>evidence/raw/bristol-city-council/src-bcc-0004_decision-notice-transport-connectivity-policy-committee-2024-09-12.pdf</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>seeded_not_downloaded</t>
+          <t>downloaded</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -381,12 +381,12 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t/>
+          <t>ce9f1e8a0682c1d935ef51f86e6976e9d8af5c353fa565bce1758eec1ff3d9b1</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
@@ -443,12 +443,12 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>sources/bristol-council/committee-packs/2024-09-12/public_reports_pack_transport_connectivity_policy_committee_2024-09-12.pdf</t>
+          <t>evidence/raw/bristol-city-council/src-bcc-0005_public-reports-pack-transport-connectivity-policy-committee-2024-09-12.pdf</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>seeded_not_downloaded</t>
+          <t>downloaded</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -458,12 +458,12 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t/>
+          <t>a5d4942ad09cd9a1b1965a624dc4553afbd3d5305d05b55f771e605a26ceab08</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
@@ -520,12 +520,12 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>sources/bristol-council/technical/feasibility/appendix_a_feasibility_study_report_wpl_scheme_bristol_final_draft.pdf</t>
+          <t>evidence/raw/bristol-city-council/src-bcc-0006_appendix-a-feasibility-study-report-wpl-scheme-bristol-final-draft.pdf</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>seeded_not_downloaded</t>
+          <t>downloaded</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -535,12 +535,12 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t/>
+          <t>92c6ff1764d64744471b348d5a3f415b486ac1973c79ba615eb248e2c95d44da</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
@@ -597,12 +597,12 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>sources/bristol-council/equalities-risk/appendix_b_eqia_workplace_parking_levy_obc_final_2024-08-20.pdf</t>
+          <t>evidence/raw/bristol-city-council/src-bcc-0007_appendix-b-eqia-workplace-parking-levy-obc-final-2024-08-20.pdf</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>seeded_not_downloaded</t>
+          <t>downloaded</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -612,12 +612,12 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t/>
+          <t>f709f37b79f74cba985c192b876131563fff8d9c732306f82b8573d54f74a03c</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
@@ -674,12 +674,12 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>sources/bristol-council/committee-reports/2025-05-15/committee_report_workplace_parking_levy_update_2025-05-15.pdf</t>
+          <t>evidence/raw/bristol-city-council/src-bcc-0008_committee-report-workplace-parking-levy-update-2025-05-15.pdf</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>seeded_not_downloaded</t>
+          <t>downloaded</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -689,12 +689,12 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t/>
+          <t>5ab6c244df2fbc7b8a470a8af314f5c17cfdcb849493fd2232af402402f1a391</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
@@ -828,12 +828,12 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>sources/bristol-council/committee-reports/2025-10-23/committee_report_wpl_october_2025.pdf</t>
+          <t>evidence/raw/bristol-city-council/src-bcc-0009_committee-report-wpl-october-2025.pdf</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>seeded_not_downloaded</t>
+          <t>downloaded</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -843,12 +843,12 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t/>
+          <t>cfdf5f4c2ac22bd3967bbf12440f3047e21db838ae1b18097caa7009170964e5</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
@@ -905,12 +905,12 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>sources/bristol-council/equalities-risk/appendix_b_eqia_workplace_parking_levy_reviewed_sept_2025.pdf</t>
+          <t>evidence/raw/bristol-city-council/src-bcc-0010_appendix-b-eqia-workplace-parking-levy-reviewed-sept-2025.pdf</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>seeded_not_downloaded</t>
+          <t>downloaded</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -920,12 +920,12 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t/>
+          <t>285a5c4d8c7c1a0a2b9748cd0d7d832df4a2d83ac729e9041dfc26ae1736a550</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
@@ -982,12 +982,12 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>sources/bristol-council/committee-packs/2025-10-23/public_reports_pack_transport_connectivity_policy_committee_2025-10-23.pdf</t>
+          <t>evidence/raw/bristol-city-council/src-bcc-0011_public-reports-pack-transport-connectivity-policy-committee-2025-10-23.pdf</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>seeded_not_downloaded</t>
+          <t>downloaded</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -997,12 +997,12 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t/>
+          <t>e56fe179eacfeba9ac04863600278c160dcafa39ef3795742648800fc5d42219</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
@@ -1213,12 +1213,12 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>sources/bristol-council/committee-reports/2026-03-19/committee_report_workplace_parking_levy_march_2026.pdf</t>
+          <t>evidence/raw/bristol-city-council/src-bcc-0014_committee-report-workplace-parking-levy-march-2026.pdf</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>seeded_not_downloaded</t>
+          <t>downloaded</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -1228,12 +1228,12 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t/>
+          <t>7c8b10d7f85111df088653065a4ccfecddfa5ec0276c8a3c8b190381e060cd82</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
@@ -1290,12 +1290,12 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>sources/bristol-council/committee-packs/2026-03-19/public_reports_pack_transport_connectivity_policy_committee_2026-03-19.pdf</t>
+          <t>evidence/raw/bristol-city-council/src-bcc-0015_public-reports-pack-transport-connectivity-policy-committee-2026-03-19.pdf</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>seeded_not_downloaded</t>
+          <t>downloaded</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
@@ -1305,12 +1305,12 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t/>
+          <t>da2f7aab9b74d0ec6a5b513f94a0c105ee87b526fef4c380a1208a1de816f1c3</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
@@ -1367,12 +1367,12 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>sources/bristol-council/forward-plans/transport_connectivity_policy_committee_forward_plan_2026-01-21.pdf</t>
+          <t>evidence/raw/bristol-city-council/src-bcc-0016_transport-connectivity-policy-committee-forward-plan-2026-01-21.pdf</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>seeded_not_downloaded</t>
+          <t>downloaded</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
@@ -1382,12 +1382,12 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t/>
+          <t>751e19a6e39e852f6937c4cd3939b8142a36f7f72382067f499482a06c0bbf20</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
@@ -1444,12 +1444,12 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>sources/bristol-council/forward-plans/transport_connectivity_policy_committee_forward_plan_update_2026-02-18.pdf</t>
+          <t>evidence/raw/bristol-city-council/src-bcc-0017_transport-connectivity-policy-committee-forward-plan-update-2026-02-18.pdf</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>seeded_not_downloaded</t>
+          <t>downloaded</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
@@ -1459,12 +1459,12 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t/>
+          <t>aea36eb0adae70292e192a9c290849b74251e46aa35dc965ce8234214764a90c</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
@@ -1598,12 +1598,12 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>sources/weca/strategy/jltp4_adopted_joint_local_transport_plan_4_2020-2036.pdf</t>
+          <t>evidence/raw/west-of-england-mca/src-weca-0001_jltp4-adopted-joint-local-transport-plan-4-2020-2036.pdf</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>seeded_not_downloaded</t>
+          <t>downloaded</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
@@ -1613,12 +1613,12 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t/>
+          <t>41f7c44dc5f63ec44af8f6a3a0a0887d42a8685c78192ddf2aee9c1d691852d0</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
@@ -1752,12 +1752,12 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>sources/weca/strategy/combined_authority_bus_strategy_updated_sept_2021.pdf</t>
+          <t>evidence/raw/west-of-england-mca/src-weca-0003_combined-authority-bus-strategy-updated-sept-2021.pdf</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>seeded_not_downloaded</t>
+          <t>downloaded</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
@@ -1767,12 +1767,12 @@
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t/>
+          <t>a80c1744fc56e56a987da7fe349451e77464fa925f2cec18aaf91824913e25b7</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
@@ -1829,12 +1829,12 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>sources/weca/strategy/west_of_england_bus_service_improvement_plan_2024.pdf</t>
+          <t>evidence/raw/west-of-england-mca/src-weca-0004_west-of-england-bus-service-improvement-plan-2024.pdf</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>seeded_not_downloaded</t>
+          <t>downloaded</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
@@ -1844,12 +1844,12 @@
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t/>
+          <t>ab5ab0f597db457bf93ff35ff3ce53075cb4e285d0d031ca9a8a9a433b43d9d7</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
@@ -1983,12 +1983,12 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>sources/weca/assurance/west_of_england_local_growth_assurance_framework_january_2024.pdf</t>
+          <t>evidence/raw/west-of-england-mca/src-weca-0006_west-of-england-local-growth-assurance-framework-january-2024.pdf</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>seeded_not_downloaded</t>
+          <t>downloaded</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
@@ -1998,12 +1998,12 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t/>
+          <t>e9e22f2870ea2a5d864d4f602e3fd2f7356506a9b86351a0f24f88072a8cc1f1</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
@@ -2368,12 +2368,12 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>sources/dft/business-case-guidance/dft_transport_business_case_guidance.html</t>
+          <t>evidence/raw/dft-and-tag/src-dft-0001_dft-transport-business-case-guidance.html</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>seeded_not_downloaded</t>
+          <t>downloaded</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
@@ -2383,12 +2383,12 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t/>
+          <t>aefbebb13963f90504293cabfcb997eb86d0ccdc4e3d37cb9fb49b89f6cdd8ef</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
@@ -2445,12 +2445,12 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>sources/statutory/transport_act_2000_explanatory_notes_road_user_charging_wpl.html</t>
+          <t>evidence/raw/legislation/src-leg-0001_transport-act-2000-explanatory-notes-road-user-charging-wpl.html</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>seeded_not_downloaded</t>
+          <t>downloaded</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
@@ -2460,12 +2460,12 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t/>
+          <t>6ff2de7f46d7713904f1e375fd40a91203b25df1439430c27b33305916262a6e</t>
         </is>
       </c>
       <c r="O32" t="inlineStr">
@@ -2522,12 +2522,12 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>sources/nottingham/annual-reports/nottingham_wpl_annual_report_2023-2024.pdf</t>
+          <t>evidence/raw/nottingham/src-nott-0001_nottingham-wpl-annual-report-2023-2024.pdf</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>seeded_not_downloaded</t>
+          <t>downloaded</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
@@ -2537,12 +2537,12 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t/>
+          <t>2e4ed5c89efcaf580741bd396138decad4fafcdbc97cc7479049ab047366deea</t>
         </is>
       </c>
       <c r="O33" t="inlineStr">
@@ -2599,12 +2599,12 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>sources/nottingham/reports/nottingham_wpl_decade_of_inspiring_growth_report.pdf</t>
+          <t>evidence/raw/nottingham/src-nott-0002_nottingham-wpl-decade-of-inspiring-growth-report.pdf</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>seeded_not_downloaded</t>
+          <t>downloaded</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
@@ -2614,12 +2614,12 @@
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t/>
+          <t>a3868b1248d442f6081ff0a69def8d0374e844ab395847559537fac9beba3517</t>
         </is>
       </c>
       <c r="O34" t="inlineStr">
@@ -2676,12 +2676,12 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>sources/nottingham/academic/dale_et_al_2017_nottingham_wpl_congestion_evaluation.pdf</t>
+          <t>evidence/raw/academic/src-academic-0001_dale-et-al-2017-nottingham-wpl-congestion-evaluation.pdf</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>seeded_not_downloaded</t>
+          <t>download_failed</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
@@ -2691,7 +2691,7 @@
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
@@ -2753,12 +2753,12 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>sources/nottingham/academic/nottingham_wpl_travel_to_work_mode_share_2019.pdf</t>
+          <t>evidence/raw/academic/src-academic-0002_nottingham-wpl-travel-to-work-mode-share-2019.pdf</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>seeded_not_downloaded</t>
+          <t>downloaded</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
@@ -2768,12 +2768,12 @@
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t/>
+          <t>b812eef4bc3b94709d0ddc6a5c1bae1476ca4d6acdafcd16c84e538e4c028715</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
@@ -3061,12 +3061,12 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>sources/uk-precedent/tfl/tfl_workplace_parking_levy_faqs_january_2020.pdf</t>
+          <t>evidence/raw/uk-comparators/src-tfl-0001_tfl-workplace-parking-levy-faqs-january-2020.pdf</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>seeded_not_downloaded</t>
+          <t>downloaded</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
@@ -3076,12 +3076,12 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t/>
+          <t>f62efc5a9719deb94d8f0cc31b8926f0c12d3c002ffd26d457f3a4a131e9eb00</t>
         </is>
       </c>
       <c r="O40" t="inlineStr">
@@ -3138,12 +3138,12 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>sources/uk-precedent/leicester/leicester_wpl_evidence_based_review_2021-05-19.pdf</t>
+          <t>evidence/raw/uk-comparators/src-uk-0003_leicester-wpl-evidence-based-review-2021-05-19.pdf</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>seeded_not_downloaded</t>
+          <t>downloaded</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
@@ -3153,12 +3153,12 @@
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t/>
+          <t>337d30947f758182652a1d7d6543eb0a7ab01054a46aa6d199653e534e682aa8</t>
         </is>
       </c>
       <c r="O41" t="inlineStr">
@@ -3472,6 +3472,1777 @@
       <c r="O45" t="inlineStr">
         <is>
           <t>Party-political source; optional and should not anchor factual claims.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>SRC-LEG-0002</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>added-primary</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>1_must</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>statutory_and_business_case</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>UK legislation</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Transport Act 2000 current contents</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>https://www.legislation.gov.uk/ukpga/2000/38/contents</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>evidence/raw/legislation/src-leg-0002_src-leg-0002-transport-act-2000-current-contents.html</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>downloaded</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>1_current_legislation</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>3b92c92cd6e87bddc07677fa4804ba6c00dc6555947f118432414cc9f14cc7b0</t>
+        </is>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>Current legislation spine for WPL powers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>SRC-LEG-0003</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>added-primary</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>1_must</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>statutory_and_business_case</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>UK legislation</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Transport Act 2000 section 184 confirmation</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>https://www.legislation.gov.uk/ukpga/2000/38/section/184</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>evidence/raw/legislation/src-leg-0003_src-leg-0003-transport-act-2000-section-184-confirmation.html</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>downloaded</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>1_current_legislation</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>598f9901a1a63d565c7f19e9cdbb6d1827b740bcbf8cc14a4cc97d78d97a0329</t>
+        </is>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>Confirmation route control.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>SRC-LEG-0004</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>added-primary</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>1_must</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>statutory_and_business_case</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>UK legislation</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Transport Act 2000 Schedule 12 net proceeds</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>https://www.legislation.gov.uk/ukpga/2000/38/schedule/12</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>evidence/raw/legislation/src-leg-0004_src-leg-0004-transport-act-2000-schedule-12-net-proceeds.html</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>downloaded</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>1_current_legislation</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>739766f35aafef854a280b891a6e1c77b466c9386bfc97a52d6b4e323d4becff</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>General plan and programme requirements for net proceeds.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>SRC-LEG-0005</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>added-primary</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>1_must</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>statutory_and_business_case</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>UK legislation</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Workplace Parking Levy (England) Regulations 2009</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>2009</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>https://www.legislation.gov.uk/uksi/2009/2085/contents</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>evidence/raw/legislation/src-leg-0005_src-leg-0005-workplace-parking-levy-england-regulations-2009.html</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>downloaded</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>1_current_legislation</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>85025ff9bda78f5e278411fda05a477147e72b556e940edc84641fb8670f8eec</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>Includes RPI-only variation exemption control.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>SRC-LEG-0006</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>added-primary</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>1_must</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>statutory_and_business_case</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>UK legislation</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Road User Charging and Workplace Parking Levy (Net Proceeds) (England) Regulations 2003</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>2003</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>https://www.legislation.gov.uk/uksi/2003/110/contents</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>evidence/raw/legislation/src-leg-0006_src-leg-0006-road-user-charging-and-workplace-parking-levy-net-proceeds-england-regulation.html</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>downloaded</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>1_current_legislation</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>2f9857f60c064b29610b96ea78edcbe46634256362cb0fa293c095c2104094dc</t>
+        </is>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>Net proceeds accounting control.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>SRC-LEG-0007</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>added-primary</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>1_must</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>statutory_and_business_case</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>UK legislation</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Road User Charging and WPL Classes of Motor Vehicles Regulations 2001</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>2001</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>https://www.legislation.gov.uk/uksi/2001/2793/contents</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>evidence/raw/legislation/src-leg-0007_src-leg-0007-road-user-charging-and-wpl-classes-of-motor-vehicles-regulations-2001.html</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>downloaded</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>1_current_legislation</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>c712a662d4961646a6a0a7da94d51f07d729ee4991fcc892b61c5ff920fedfe0</t>
+        </is>
+      </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>Vehicle class control.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>SRC-LEG-0008</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>added-primary</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>1_must</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>statutory_and_business_case</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>UK legislation</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Road Traffic Regulation Act 1984 section 121A</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>https://www.legislation.gov.uk/ukpga/1984/27/section/121A</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>evidence/raw/legislation/src-leg-0008_src-leg-0008-road-traffic-regulation-act-1984-section-121a.html</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>downloaded</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>1_current_legislation</t>
+        </is>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>3e368e8b18ad54be8d3a687468992b7a89d0707395ab182c17900ec2edfbf6a9</t>
+        </is>
+      </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>Local traffic authority definition control.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>SRC-LEG-0009</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>added-primary</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>1_must</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>weca_context</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>UK legislation</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>West of England Combined Authority Order 2017</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>https://www.legislation.gov.uk/uksi/2017/126/contents</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>evidence/raw/legislation/src-leg-0009_src-leg-0009-west-of-england-combined-authority-order-2017.html</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>downloaded</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>1_current_legislation</t>
+        </is>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>679a172f7fed254a9426a478bac67a417574439ecc3da1a34f6cdd8dec7df3b4</t>
+        </is>
+      </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>WECA/MCA transport-function verification.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>SRC-LEG-0010</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>added-primary</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>1_must</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>weca_context</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>UK legislation</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>SI 2026/519 regulation 29</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>https://www.legislation.gov.uk/uksi/2026/519/regulation/29</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>evidence/raw/legislation/src-leg-0010_src-leg-0010-si-2026-519-regulation-29.html</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>downloaded</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>1_current_legislation</t>
+        </is>
+      </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>7321ad0d149e0acecd44b4375db2d40c50b3349182f59a1d45a97543995c6e09</t>
+        </is>
+      </c>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>Potential WECA/MCA current-law change flagged by discovery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>SRC-HMT-0001</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>added-primary</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>1_must</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>statutory_and_business_case</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>HM Treasury</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>The Green Book 2026</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>https://www.gov.uk/government/publications/the-green-book-appraisal-and-evaluation-in-central-government/the-green-book-2026</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>evidence/raw/hm-treasury/src-hmt-0001_src-hmt-0001-the-green-book-2026.html</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>downloaded</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>2_official_government_guidance</t>
+        </is>
+      </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>ce2a23f36a003706307f93ca03fea699115469784f11f7c54c7de7c66b9c2212</t>
+        </is>
+      </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>Current Green Book metrics and appraisal controls.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>SRC-HMT-0002</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>added-primary</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>1_must</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>statutory_and_business_case</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>HM Treasury</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>The Magenta Book</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>https://www.gov.uk/government/publications/the-magenta-book</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>evidence/raw/hm-treasury/src-hmt-0002_src-hmt-0002-the-magenta-book.html</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>downloaded</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>2_official_government_guidance</t>
+        </is>
+      </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>5fbf8ea170ddeb22f470a42e689caa03e6369460538fa3fb07c78f43e4f7fa43</t>
+        </is>
+      </c>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>Evaluation guidance control.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>SRC-HMT-0003</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>added-primary</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>1_must</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>statutory_and_business_case</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>HM Treasury</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Managing Public Money</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>https://www.gov.uk/government/publications/managing-public-money</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>evidence/raw/hm-treasury/src-hmt-0003_src-hmt-0003-managing-public-money.html</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>downloaded</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>2_official_government_guidance</t>
+        </is>
+      </c>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>dfac3771439f193c1c5312fae4a675543d873aff4c82c7d7ef99e46156b9a2f8</t>
+        </is>
+      </c>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>Public money control.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>SRC-HMT-0004</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>added-primary</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>1_must</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>statutory_and_business_case</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>HM Treasury</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>The Aqua Book</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>https://www.gov.uk/government/publications/the-aqua-book-guidance-on-producing-quality-analysis-for-government</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>evidence/raw/hm-treasury/src-hmt-0004_src-hmt-0004-the-aqua-book.html</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>downloaded</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>2_official_government_guidance</t>
+        </is>
+      </c>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="N58" t="inlineStr">
+        <is>
+          <t>f4acfa1e3b4eba3204de20973dc1f8597c528f96f40faa17b04e2b3f3242cd30</t>
+        </is>
+      </c>
+      <c r="O58" t="inlineStr">
+        <is>
+          <t>Analytical assurance control.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>SRC-DFT-0002</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>added-primary</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>1_must</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>statutory_and_business_case</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Department for Transport</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Transport analysis guidance</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>https://www.gov.uk/guidance/transport-analysis-guidance</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>evidence/raw/dft-and-tag/src-dft-0002_src-dft-0002-transport-analysis-guidance.html</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>downloaded</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>2_official_government_guidance</t>
+        </is>
+      </c>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t>a88f93e9dec4042c17bbd8b0b2e41a0635a3452667f95beaf5235f9c6272df7e</t>
+        </is>
+      </c>
+      <c r="O59" t="inlineStr">
+        <is>
+          <t>TAG landing page and current update control.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>SRC-LEG-0011</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>added-primary</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>1_must</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>statutory_and_business_case</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>UK legislation</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Workplace Parking Levy (England) Regulations 2009 whole instrument</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>2009</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>https://www.legislation.gov.uk/uksi/2009/2085/made</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>evidence/raw/legislation/src-leg-0011_src-leg-0011-workplace-parking-levy-england-regulations-2009-whole-instrument.html</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>downloaded</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>1_current_legislation</t>
+        </is>
+      </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>ffc8c37e5742cdaa5b984802f57c96fd29fcb41f3d690a9d67c32c5a90ef5d7e</t>
+        </is>
+      </c>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t>Whole-instrument text for confirmation exemption, licensing charges and penalty enforcement controls.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>SRC-LEG-0012</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>added-primary</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>1_must</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>statutory_and_business_case</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>UK legislation</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Road User Charging and WPL Net Proceeds Regulations 2003 whole instrument</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>2003</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>https://www.legislation.gov.uk/uksi/2003/110/made</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>evidence/raw/legislation/src-leg-0012_src-leg-0012-road-user-charging-and-wpl-net-proceeds-regulations-2003-whole-instrument.html</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>downloaded</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>1_current_legislation</t>
+        </is>
+      </c>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="N61" t="inlineStr">
+        <is>
+          <t>71361b878bfffea1e1da8c1624b65e437eff89f28b088c6b15935114e9795755</t>
+        </is>
+      </c>
+      <c r="O61" t="inlineStr">
+        <is>
+          <t>Whole-instrument text for net proceeds accounting and deductions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>SRC-LEG-0013</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>added-primary</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>1_must</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>statutory_and_business_case</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>UK legislation</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Road User Charging and WPL Classes of Motor Vehicles Regulations 2001 whole instrument</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>2001</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>https://www.legislation.gov.uk/uksi/2001/2793/made</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>evidence/raw/legislation/src-leg-0013_src-leg-0013-road-user-charging-and-wpl-classes-of-motor-vehicles-regulations-2001-whole-i.html</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>downloaded</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>1_current_legislation</t>
+        </is>
+      </c>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="N62" t="inlineStr">
+        <is>
+          <t>c7f1a31c57abdcba332517da201a369fba81fd9117fe0dc0a5c84e06cb489dd6</t>
+        </is>
+      </c>
+      <c r="O62" t="inlineStr">
+        <is>
+          <t>Whole-instrument text for vehicle-class controls relevant to any licensing scheme exclusions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>SRC-BCC-0022</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>added-primary</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>1_must</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>bristol_governance</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Bristol City Council - Transport and Connectivity Policy Committee</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Printed minutes - Transport and Connectivity Policy Committee 12 September 2024</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>2024-09-12</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>https://democracy.bristol.gov.uk/documents/g11272/Printed%20minutes%2012th-Sep-2024%2017.00%20Transport%20Connectivity%20Policy%20Committee.pdf?T=1</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>evidence/raw/bristol-city-council/src-bcc-0022_src-bcc-0022-printed-minutes-transport-and-connectivity-policy-committee-12-september-2024.pdf</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>downloaded</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>3_formal_public_body_source</t>
+        </is>
+      </c>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="N63" t="inlineStr">
+        <is>
+          <t>dfb02c8d90752208c124fd57cf8874875c09caceeca9ebfbedc15cb676b356bd</t>
+        </is>
+      </c>
+      <c r="O63" t="inlineStr">
+        <is>
+          <t>Minutes companion to the September 2024 WPL Stage One Development decision.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>SRC-BCC-0023</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>added-primary</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>1_must</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>bristol_governance</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Bristol City Council - Transport and Connectivity Policy Committee</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Decision notice - Transport and Connectivity Policy Committee 23 October 2025</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>2025-10-23</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>https://democracy.bristol.gov.uk/documents/g11586/Decisions%2023rd-Oct-2025%2017.00%20Transport%20Connectivity%20Policy%20Committee.pdf?T=2</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>evidence/raw/bristol-city-council/src-bcc-0023_src-bcc-0023-decision-notice-transport-and-connectivity-policy-committee-23-october-2025.pdf</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>downloaded</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>3_formal_public_body_source</t>
+        </is>
+      </c>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="N64" t="inlineStr">
+        <is>
+          <t>67b6a9efb1f96f2e85fcd4c3930b9d180a526283e941b687cf7ead6bceccc28e</t>
+        </is>
+      </c>
+      <c r="O64" t="inlineStr">
+        <is>
+          <t>Decision notice needed to distinguish October 2025 WPL update from formal approval.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>SRC-BCC-0024</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>added-primary</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>1_must</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>bristol_governance</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Bristol City Council - Transport and Connectivity Policy Committee</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Printed minutes - Transport and Connectivity Policy Committee 23 October 2025</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>2025-10-23</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>https://democracy.bristol.gov.uk/documents/g11586/Printed%20minutes%2023rd-Oct-2025%2017.00%20Transport%20Connectivity%20Policy%20Committee.pdf?T=1</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>evidence/raw/bristol-city-council/src-bcc-0024_src-bcc-0024-printed-minutes-transport-and-connectivity-policy-committee-23-october-2025.pdf</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>downloaded</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>3_formal_public_body_source</t>
+        </is>
+      </c>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="N65" t="inlineStr">
+        <is>
+          <t>ec4b1da46a4cb941cfbf76ed11bc15c06ea7f622aeb214b00668445a89e04396</t>
+        </is>
+      </c>
+      <c r="O65" t="inlineStr">
+        <is>
+          <t>Minutes companion for October 2025 WPL update meeting.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>SRC-BCC-0025</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>added-primary</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>1_must</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>bristol_governance</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Bristol City Council - Transport and Connectivity Policy Committee</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Decision notice - Transport and Connectivity Policy Committee 19 March 2026</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>https://democracy.bristol.gov.uk/documents/g11589/Decisions%2019th-Mar-2026%2017.00%20Transport%20Connectivity%20Policy%20Committee.pdf?T=2</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>evidence/raw/bristol-city-council/src-bcc-0025_src-bcc-0025-decision-notice-transport-and-connectivity-policy-committee-19-march-2026.pdf</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>downloaded</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>3_formal_public_body_source</t>
+        </is>
+      </c>
+      <c r="M66" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="N66" t="inlineStr">
+        <is>
+          <t>47cf5ed46599beedb6cd9f3b30a3f3481df041536c212231e11083c02852de0f</t>
+        </is>
+      </c>
+      <c r="O66" t="inlineStr">
+        <is>
+          <t>Decision notice needed to verify March 2026 WPL update status.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>SRC-BCC-0026</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>added-primary</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>1_must</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>bristol_governance</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Bristol City Council - Transport and Connectivity Policy Committee</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Printed minutes - Transport and Connectivity Policy Committee 19 March 2026</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>https://democracy.bristol.gov.uk/documents/g11589/Printed%20minutes%2019th-Mar-2026%2017.00%20Transport%20Connectivity%20Policy%20Committee.pdf?T=1</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>evidence/raw/bristol-city-council/src-bcc-0026_src-bcc-0026-printed-minutes-transport-and-connectivity-policy-committee-19-march-2026.pdf</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>downloaded</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>3_formal_public_body_source</t>
+        </is>
+      </c>
+      <c r="M67" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="N67" t="inlineStr">
+        <is>
+          <t>6fde2cb7fc67be69e76fa12d902afe8b3f7f505ff535fef4df28ea53801edb06</t>
+        </is>
+      </c>
+      <c r="O67" t="inlineStr">
+        <is>
+          <t>Minutes companion for March 2026 WPL update meeting.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>SRC-BCC-0027</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>added-primary</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>1_must</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>equalities_and_risk</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Bristol City Council</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Appendix B - Equality Impact Assessment - Workplace Parking Levy reviewed Oct 2025</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>https://democracy.bristol.gov.uk/documents/s124298/Appendix%20B%20-%20Equality%20Impact%20Assessment%20-%20Workplace%20Parking%20Levy%20reviewed%20Oct%202025.pdf</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>evidence/raw/bristol-city-council/src-bcc-0027_src-bcc-0027-appendix-b-equality-impact-assessment-workplace-parking-levy-reviewed-oct-202.pdf</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>downloaded</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>3_formal_public_body_source</t>
+        </is>
+      </c>
+      <c r="M68" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="N68" t="inlineStr">
+        <is>
+          <t>ca2f18fb67e45bcaaa3bf75d2174587833575ac93b26c7dae62f7b49d6a1e889</t>
+        </is>
+      </c>
+      <c r="O68" t="inlineStr">
+        <is>
+          <t>March 2026 pack lists this as an EqIA appendix; compare with August 2024 and September 2025 EqIAs.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: add Stage 2 legal governance baseline
</commit_message>
<xml_diff>
--- a/evidence/source_register.xlsx
+++ b/evidence/source_register.xlsx
@@ -2455,7 +2455,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>1_current_legislation</t>
+          <t>2_official_government_guidance</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -2470,7 +2470,7 @@
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>Use with legislation text if a deeper legal section is needed.</t>
+          <t>Official explanatory notes; use with current legislation text and do not treat as current amended legislation.</t>
         </is>
       </c>
     </row>
@@ -3302,7 +3302,7 @@
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>3_formal_public_body_source</t>
+          <t>7_professional_or_context_source</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
@@ -3379,7 +3379,7 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>3_formal_public_body_source</t>
+          <t>7_professional_or_context_source</t>
         </is>
       </c>
       <c r="M44" t="inlineStr">
@@ -3456,7 +3456,7 @@
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>3_formal_public_body_source</t>
+          <t>7_professional_or_context_source</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">

</xml_diff>

<commit_message>
docs: refine Stage 2 governance evidence
</commit_message>
<xml_diff>
--- a/evidence/source_register.xlsx
+++ b/evidence/source_register.xlsx
@@ -1198,7 +1198,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1238,7 +1238,7 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>Primary source for current status as at March 2026.</t>
+          <t>Primary source for current status as at the 19 March 2026 committee meeting.</t>
         </is>
       </c>
     </row>
@@ -2060,12 +2060,12 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>sources/weca/assurance/west_of_england_local_growth_assurance_framework_july_2025_final.pdf</t>
+          <t>evidence/raw/west-of-england-mca/src-weca-0007_west-of-england-local-growth-assurance-framework-july-2025-final.pdf</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>seeded_not_downloaded</t>
+          <t>downloaded</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
@@ -2075,17 +2075,17 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t/>
+          <t>2f13666fc5302e915d933dc3415385682183c7b820262e21b1a3941b9af28b00</t>
         </is>
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>Use for future-facing OBC/FBC governance, but be careful about dates when analysing earlier decisions.</t>
+          <t>Current WECA assurance framework for possible MCA funding/assurance route; not WPL consent or approval evidence.</t>
         </is>
       </c>
     </row>
@@ -5243,6 +5243,1931 @@
       <c r="O68" t="inlineStr">
         <is>
           <t>March 2026 pack lists this as an EqIA appendix; compare with August 2024 and September 2025 EqIAs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>SRC-BCC-0028</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>added-primary</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>1_must</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>bristol_governance</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Bristol City Council</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>Bristol City Council Constitution page</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>current_webpage</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>https://www.bristol.gov.uk/council/how-council-decisions-are-made/constitution</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>evidence/raw/bristol-city-council/src-bcc-0028_bristol-city-council-constitution-page.html</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>downloaded</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>3_formal_public_body_source</t>
+        </is>
+      </c>
+      <c r="M69" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="N69" t="inlineStr">
+        <is>
+          <t>863ffd1d7121910360ef44c75c1239c9e3c0ad17e0cc63c46844d23467413cc9</t>
+        </is>
+      </c>
+      <c r="O69" t="inlineStr">
+        <is>
+          <t>Official index page for current Bristol constitution and officer scheme of delegations; use to locate source PDFs, not to infer WPL powers by itself.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>SRC-BCC-0029</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>added-primary</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>1_must</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>bristol_governance</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Bristol City Council - Constitution</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Part 3.2 - Terms of Reference of Committees</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>2025-11</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>https://democracy.bristol.gov.uk/documents/s125434/Part%203.2%20-%20Terms%20of%20Reference%20of%20Committees%20-%20November%202025.pdf</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>evidence/raw/bristol-city-council/src-bcc-0029_part-3-2-terms-of-reference-of-committees-november-2025.pdf</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>downloaded</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>3_formal_public_body_source</t>
+        </is>
+      </c>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="N70" t="inlineStr">
+        <is>
+          <t>0376766267747a33131d95c4593073f45cc18e16141432b8257accd9a73bce59</t>
+        </is>
+      </c>
+      <c r="O70" t="inlineStr">
+        <is>
+          <t>Current constitution source for committee remits; review for Transport and Connectivity Committee decision route.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>SRC-BCC-0030</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>added-primary</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>1_must</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>bristol_governance</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Bristol City Council - Constitution</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>Part 3.4 - Delegations to Officers</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>https://democracy.bristol.gov.uk/documents/s125436/Part%203.4%20-%20Delegations%20to%20Officers%20-%20January%202026.pdf</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>evidence/raw/bristol-city-council/src-bcc-0030_part-3-4-delegations-to-officers-january-2026.pdf</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>downloaded</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>3_formal_public_body_source</t>
+        </is>
+      </c>
+      <c r="M71" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="N71" t="inlineStr">
+        <is>
+          <t>fb980700ba5696561fea6a361a8ee716b2dbe6ebed9ef6736f11434873db3c2f</t>
+        </is>
+      </c>
+      <c r="O71" t="inlineStr">
+        <is>
+          <t>Current constitution source for officer delegations; must be read with directorate-specific Growth and Regeneration scheme.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>SRC-BCC-0031</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>added-primary</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>1_must</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>bristol_governance</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Bristol City Council</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Officer Scheme of Delegation - Growth and Regeneration</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>https://www.bristol.gov.uk/files/documents/7693-scheme-of-delegation-growth-and-regeneration</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>evidence/raw/bristol-city-council/src-bcc-0031_officer-scheme-of-delegation-growth-and-regeneration.pdf</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>downloaded</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>3_formal_public_body_source</t>
+        </is>
+      </c>
+      <c r="M72" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="N72" t="inlineStr">
+        <is>
+          <t>527f89ce9b199a9ec552999d1d2ca0a2d5d8988060657ffcddb7ce4f571450dd</t>
+        </is>
+      </c>
+      <c r="O72" t="inlineStr">
+        <is>
+          <t>Directorate delegation source for Executive Director Growth and Regeneration; fetched PDF states approved/published June 2026; relevant because WPL Stage One contract delegations use this officer route.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>SRC-WECA-0011</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>added-primary</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>1_must</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>weca_context</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>West of England Combined Authority</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>West of England Combined Authority Constitution page</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>current_webpage</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>https://www.westofengland-ca.gov.uk/about-us/democracy-funding-transparency/constitution/</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>evidence/raw/west-of-england-mca/src-weca-0011_west-of-england-combined-authority-constitution-page.html</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>downloaded</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>3_formal_public_body_source</t>
+        </is>
+      </c>
+      <c r="M73" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="N73" t="inlineStr">
+        <is>
+          <t>30b7c9eab7507319cf5e7b727cef0cf87ba2b4672ee49e6ea89cac9306126184</t>
+        </is>
+      </c>
+      <c r="O73" t="inlineStr">
+        <is>
+          <t>Official WECA constitution landing page linking to ModernGov constitution pack.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>SRC-WECA-0012</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>added-primary</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>1_must</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>weca_context</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>West of England Combined Authority - Constitution</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Part A Constitution</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>https://westofengland-ca.moderngov.co.uk/documents/s10989/Part%20A%20Constitution%20-%20Oct%202025%201.1.pdf</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>evidence/raw/west-of-england-mca/src-weca-0012_part-a-constitution-october-2025.pdf</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>downloaded</t>
+        </is>
+      </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>3_formal_public_body_source</t>
+        </is>
+      </c>
+      <c r="M74" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="N74" t="inlineStr">
+        <is>
+          <t>bd70210c6521652649df1a6d713967ef4e453c223e5a6acdb8f45fd5e23ca8d0</t>
+        </is>
+      </c>
+      <c r="O74" t="inlineStr">
+        <is>
+          <t>WECA constitutional framework source; use with current legislation and Part B before any role conclusion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>SRC-WECA-0013</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>added-primary</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>1_must</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>weca_context</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>West of England Combined Authority - Constitution</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>Part B Constitution - 2026 Revision</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>https://westofengland-ca.moderngov.co.uk/documents/s11374/Part%20B%20-%202026%20Revision.pdf</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>evidence/raw/west-of-england-mca/src-weca-0013_part-b-constitution-2026-revision.pdf</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>downloaded</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>3_formal_public_body_source</t>
+        </is>
+      </c>
+      <c r="M75" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="N75" t="inlineStr">
+        <is>
+          <t>914cdc865a5e8ecc914b5746cc7efdd7541ec832071cc5aa834613036ae294f4</t>
+        </is>
+      </c>
+      <c r="O75" t="inlineStr">
+        <is>
+          <t>WECA procedure, delegation and scheme-detail source; must be mapped before consent/no-role conclusions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>SRC-LEG-0014</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>added-primary</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>1_must</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>weca_context</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>UK legislation</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>English Devolution and Community Empowerment Act 2026 consequential regulations whole instrument</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>https://www.legislation.gov.uk/uksi/2026/519/made</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>evidence/raw/legislation/src-leg-0014_english-devolution-community-empowerment-consequential-regulations-2026-whole-instrument.html</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>downloaded</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>1_current_legislation</t>
+        </is>
+      </c>
+      <c r="M76" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="N76" t="inlineStr">
+        <is>
+          <t>9caca4522435638fe134ebb6e34974585b697595d38a9ac5771fa47d338dca2c</t>
+        </is>
+      </c>
+      <c r="O76" t="inlineStr">
+        <is>
+          <t>Whole consequential instrument; use with regulation 29 and current combined-authority function mapping.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>SRC-LEG-0015</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>added-primary</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>1_must</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>weca_context</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>UK legislation</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>English Devolution and Community Empowerment Act 2026 Schedule 9</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>https://www.legislation.gov.uk/ukpga/2026/23/schedule/9/enacted</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>evidence/raw/legislation/src-leg-0015_english-devolution-community-empowerment-act-2026-schedule-9.html</t>
+        </is>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>downloaded</t>
+        </is>
+      </c>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>1_current_legislation</t>
+        </is>
+      </c>
+      <c r="M77" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="N77" t="inlineStr">
+        <is>
+          <t>9fa9a5a70ceb8d3c6d21aa654996e9634b8a09df0929be123815e40a02611c61</t>
+        </is>
+      </c>
+      <c r="O77" t="inlineStr">
+        <is>
+          <t>Schedule 9 covers charges payable by undertakers executing works in maintainable highways. Not a WPL power source; retain only to avoid misclassifying it as WECA/MCA WPL authority.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>SRC-BCC-0032</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>added-primary</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>1_must</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>bristol_governance</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Bristol City Council - Constitution</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>Part 2 - Articles of the Constitution</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>2024-06</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>https://democracy.bristol.gov.uk/documents/s125432/Part%202%20-%20Articles%20-%20June%202024.pdf</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>evidence/raw/bristol-city-council/src-bcc-0032_part-2-articles-of-the-constitution-june-2024.pdf</t>
+        </is>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>downloaded</t>
+        </is>
+      </c>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>3_formal_public_body_source</t>
+        </is>
+      </c>
+      <c r="M78" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="N78" t="inlineStr">
+        <is>
+          <t>d995abe937a4e09f2992263345f9477d7a8ce2aca50db3de81d176b3193ec512</t>
+        </is>
+      </c>
+      <c r="O78" t="inlineStr">
+        <is>
+          <t>Defines key decisions and Policy Committee decision framework.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>SRC-BCC-0033</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>added-primary</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>1_must</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>bristol_governance</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Bristol City Council - Constitution</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>Part 3.1 - Full Council Functions</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>2024-05</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>https://democracy.bristol.gov.uk/documents/s125433/Part%203.1%20-%20Full%20Council%20Functions%20-%20May%202024.pdf</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>evidence/raw/bristol-city-council/src-bcc-0033_part-3-1-full-council-functions-may-2024.pdf</t>
+        </is>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>downloaded</t>
+        </is>
+      </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>3_formal_public_body_source</t>
+        </is>
+      </c>
+      <c r="M79" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="N79" t="inlineStr">
+        <is>
+          <t>ee8f3238dd4db87484fd31b5924f32cb77abec741e33191a3ca86547f5554c98</t>
+        </is>
+      </c>
+      <c r="O79" t="inlineStr">
+        <is>
+          <t>Reserved Full Council functions check for WPL decision routing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>SRC-BCC-0034</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>added-primary</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>1_must</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>bristol_governance</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Bristol City Council - Constitution</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>Part 4.2 - Access to Information Procedure Rules</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>2024-05</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>https://democracy.bristol.gov.uk/documents/s125439/Part%204.2%20-%20Access%20to%20information%20procedure%20rules%20-%20May2024.pdf</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>evidence/raw/bristol-city-council/src-bcc-0034_part-4-2-access-to-information-procedure-rules-may-2024.pdf</t>
+        </is>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>downloaded</t>
+        </is>
+      </c>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>3_formal_public_body_source</t>
+        </is>
+      </c>
+      <c r="M80" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="N80" t="inlineStr">
+        <is>
+          <t>76f242507cbd4eaa9c9d3dfff8517ef9dd829528f8aa36dac6f0fadeb5acb181</t>
+        </is>
+      </c>
+      <c r="O80" t="inlineStr">
+        <is>
+          <t>Forward plan and key-decision procedure rules.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>SRC-BCC-0035</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>added-primary</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>1_must</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>bristol_governance</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Bristol City Council - Transport and Connectivity Policy Committee</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>Decision notice - Transport and Connectivity Policy Committee 15 May 2025</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>2025-05-15</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>https://democracy.bristol.gov.uk/documents/g11583/Decisions%2015th-May-2025%2016.30%20Transport%20Connectivity%20Policy%20Committee.pdf?T=2</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>evidence/raw/bristol-city-council/src-bcc-0035_decision-notice-transport-and-connectivity-policy-committee-15-may-2025.pdf</t>
+        </is>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>downloaded</t>
+        </is>
+      </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>3_formal_public_body_source</t>
+        </is>
+      </c>
+      <c r="M81" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="N81" t="inlineStr">
+        <is>
+          <t>b962cff27418de8b231df9ea1d5297e2bce6096b7975b2644c4384969a3dbc62</t>
+        </is>
+      </c>
+      <c r="O81" t="inlineStr">
+        <is>
+          <t>Decision notice confirming WPL item was noted as an update.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>SRC-BCC-0036</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>added-primary</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>1_must</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>bristol_governance</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Bristol City Council - Transport and Connectivity Policy Committee</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>Printed minutes - Transport and Connectivity Policy Committee 15 May 2025</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>2025-05-15</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>https://democracy.bristol.gov.uk/documents/g11583/Printed%20minutes%2015th-May-2025%2016.30%20Transport%20Connectivity%20Policy%20Committee.pdf?T=1</t>
+        </is>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>evidence/raw/bristol-city-council/src-bcc-0036_printed-minutes-transport-and-connectivity-policy-committee-15-may-2025.pdf</t>
+        </is>
+      </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>downloaded</t>
+        </is>
+      </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>3_formal_public_body_source</t>
+        </is>
+      </c>
+      <c r="M82" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="N82" t="inlineStr">
+        <is>
+          <t>ca4697b7502d206060b76a69bc243b7b40335d6dfda4bf764dda6b7da4762387</t>
+        </is>
+      </c>
+      <c r="O82" t="inlineStr">
+        <is>
+          <t>Minutes confirming no WPL decision was taken and update was noted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>SRC-LEG-0016</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>added-primary</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>1_must</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>weca_context</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>UK legislation</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>English Devolution and Community Empowerment Act 2026 section 2</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>https://www.legislation.gov.uk/ukpga/2026/23/section/2/enacted</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>evidence/raw/legislation/src-leg-0016_english-devolution-community-empowerment-act-2026-section-2.html</t>
+        </is>
+      </c>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>downloaded</t>
+        </is>
+      </c>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>1_current_legislation</t>
+        </is>
+      </c>
+      <c r="M83" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="N83" t="inlineStr">
+        <is>
+          <t>9f0b50e5e611ce4014ef358240a2eabf4760508a0b7791e3862a74965326ebe7</t>
+        </is>
+      </c>
+      <c r="O83" t="inlineStr">
+        <is>
+          <t>Strategic authority areas-of-competence source; use for current-law mapping, not as WPL-specific authority by itself.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>SRC-WECA-0014</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>added-primary</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>2_should</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>weca_context</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>West of England Combined Authority</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>Transport page</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>current_webpage</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>https://www.westofengland-ca.gov.uk/what-we-do/transport/</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>evidence/raw/west-of-england-mca/src-weca-0014_weca-transport-page.html</t>
+        </is>
+      </c>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>downloaded</t>
+        </is>
+      </c>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>3_formal_public_body_source</t>
+        </is>
+      </c>
+      <c r="M84" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="N84" t="inlineStr">
+        <is>
+          <t>59ba1cf1c3c1e70fbd8fb5e35bca56f55137454107b8906f09ad25934d360d45</t>
+        </is>
+      </c>
+      <c r="O84" t="inlineStr">
+        <is>
+          <t>Public regional transport narrative; not statutory WPL authority.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>SRC-WECA-0015</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>added-primary</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>2_should</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>weca_governance</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>West of England Combined Authority</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>Combined Authority Committee details</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>current_webpage</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>https://westofengland-ca.moderngov.co.uk/mgCommitteeDetails.aspx?ID=141</t>
+        </is>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>evidence/raw/west-of-england-mca/src-weca-0015_combined-authority-committee-details.html</t>
+        </is>
+      </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>downloaded</t>
+        </is>
+      </c>
+      <c r="L85" t="inlineStr">
+        <is>
+          <t>3_formal_public_body_source</t>
+        </is>
+      </c>
+      <c r="M85" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="N85" t="inlineStr">
+        <is>
+          <t>161157444d2fff6d2aa303fd87431fb34ca2146ab6cd499bc14b921b1c943a0d</t>
+        </is>
+      </c>
+      <c r="O85" t="inlineStr">
+        <is>
+          <t>Committee-route mapping source; no WPL-specific decision located.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>SRC-WECA-0016</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>added-primary</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>2_should</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>weca_governance</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>West of England Combined Authority</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>Joint Committee details</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>current_webpage</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>https://westofengland-ca.moderngov.co.uk/mgCommitteeDetails.aspx?ID=142</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>evidence/raw/west-of-england-mca/src-weca-0016_joint-committee-details.html</t>
+        </is>
+      </c>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>downloaded</t>
+        </is>
+      </c>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>3_formal_public_body_source</t>
+        </is>
+      </c>
+      <c r="M86" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="N86" t="inlineStr">
+        <is>
+          <t>6adaeb70294fd03f60cc87776e45ecfc505aa87e3cd2c84c122e58ed71a2688a</t>
+        </is>
+      </c>
+      <c r="O86" t="inlineStr">
+        <is>
+          <t>Joint Committee route and North Somerset/legacy context source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>SRC-LEG-0017</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>added-primary</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>1_must</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>statutory_and_business_case</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>UK legislation</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>Transport Act 2000 section 178 workplace parking levy licensing schemes</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>https://www.legislation.gov.uk/ukpga/2000/38/section/178</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>evidence/raw/legislation/src-leg-0017_transport-act-2000-section-178-workplace-parking-levy-licensing-schemes.html</t>
+        </is>
+      </c>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>downloaded</t>
+        </is>
+      </c>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>1_current_legislation</t>
+        </is>
+      </c>
+      <c r="M87" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="N87" t="inlineStr">
+        <is>
+          <t>b11c6758446f9f123dc464ef02f5dac3c0af0717cce1f3db04c0085f0e729b08</t>
+        </is>
+      </c>
+      <c r="O87" t="inlineStr">
+        <is>
+          <t>Direct WPL licensing-scheme authority text.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>SRC-LEG-0018</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>added-primary</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>1_must</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>statutory_and_business_case</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>UK legislation</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>Transport Act 2000 section 179 licensing schemes made by local traffic authorities</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>https://www.legislation.gov.uk/ukpga/2000/38/section/179</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>evidence/raw/legislation/src-leg-0018_transport-act-2000-section-179-licensing-schemes-local-traffic-authorities.html</t>
+        </is>
+      </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>downloaded</t>
+        </is>
+      </c>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>1_current_legislation</t>
+        </is>
+      </c>
+      <c r="M88" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="N88" t="inlineStr">
+        <is>
+          <t>3e212ea0547c342395698380a14a6a4f92b068fa3a8144b2f69bdd8d1c4d1ac1</t>
+        </is>
+      </c>
+      <c r="O88" t="inlineStr">
+        <is>
+          <t>Direct source for authority/joint-scheme wording; must be mapped to Bristol/WECA current law.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>SRC-LEG-0019</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>added-primary</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>1_must</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>statutory_and_business_case</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>UK legislation</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>Transport Act 2000 section 180 persons liable to charges</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>https://www.legislation.gov.uk/ukpga/2000/38/section/180</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>evidence/raw/legislation/src-leg-0019_transport-act-2000-section-180-persons-liable-to-charges.html</t>
+        </is>
+      </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>downloaded</t>
+        </is>
+      </c>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>1_current_legislation</t>
+        </is>
+      </c>
+      <c r="M89" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="N89" t="inlineStr">
+        <is>
+          <t>1cbe96f20325ef1133e11be10f1eeeda98afcf865a4b245acb41b2c500c4dfe0</t>
+        </is>
+      </c>
+      <c r="O89" t="inlineStr">
+        <is>
+          <t>Direct WPL liability source for licensing and scheme design controls.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>SRC-LEG-0020</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>added-primary</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>1_must</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>statutory_and_business_case</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>UK legislation</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>Transport Act 2000 section 198 interpretation of local transport policies</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>https://www.legislation.gov.uk/ukpga/2000/38/section/198</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>evidence/raw/legislation/src-leg-0020_transport-act-2000-section-198-interpretation-local-transport-policies.html</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>downloaded</t>
+        </is>
+      </c>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>1_current_legislation</t>
+        </is>
+      </c>
+      <c r="M90" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="N90" t="inlineStr">
+        <is>
+          <t>57ef53c4677e7c62cd98d28a1f05be09f1a2646cee84e05e4e4cbf0b287164d7</t>
+        </is>
+      </c>
+      <c r="O90" t="inlineStr">
+        <is>
+          <t>Direct interpretation source for local transport policies in WPL statutory context.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>SRC-LEG-0021</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>added-primary</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>1_must</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>statutory_and_business_case</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>UK legislation</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>Transport Act 2000 section 108 local transport plans</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>https://www.legislation.gov.uk/ukpga/2000/38/section/108</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>evidence/raw/legislation/src-leg-0021_transport-act-2000-section-108-local-transport-plans.html</t>
+        </is>
+      </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>downloaded</t>
+        </is>
+      </c>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>1_current_legislation</t>
+        </is>
+      </c>
+      <c r="M91" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="N91" t="inlineStr">
+        <is>
+          <t>0905aefa70014fcf3440f11ddf0520650ce3812ff07e8b06c20daf637ea35e39</t>
+        </is>
+      </c>
+      <c r="O91" t="inlineStr">
+        <is>
+          <t>Local transport plan context source; map carefully after 2026 devolution amendments.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>SRC-LEG-0022</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>added-primary</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>1_must</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>weca_context</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>UK legislation</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>West of England Combined Authority Order 2017 article 7 current revised text</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>https://www.legislation.gov.uk/uksi/2017/126/article/7</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>evidence/raw/legislation/src-leg-0022_weca-order-2017-article-7-current.html</t>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>downloaded</t>
+        </is>
+      </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>1_current_legislation</t>
+        </is>
+      </c>
+      <c r="M92" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="N92" t="inlineStr">
+        <is>
+          <t>729db0c6fb5f5dfc1acf788c6b9876305195fa0236a021ce489d2b67fa011211</t>
+        </is>
+      </c>
+      <c r="O92" t="inlineStr">
+        <is>
+          <t>Direct current revised article source for WECA Order function mapping after 2026 amendments.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>SRC-LEG-0023</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>added-primary</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>1_must</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>weca_context</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>UK legislation</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>West of England Combined Authority Order 2017 article 8 current revised text</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>https://www.legislation.gov.uk/uksi/2017/126/article/8</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>evidence/raw/legislation/src-leg-0023_weca-order-2017-article-8-current.html</t>
+        </is>
+      </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>downloaded</t>
+        </is>
+      </c>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>1_current_legislation</t>
+        </is>
+      </c>
+      <c r="M93" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="N93" t="inlineStr">
+        <is>
+          <t>12fba6435a178ba6684c8b5e738d44da633568a5bf301055f4672303bda3257d</t>
+        </is>
+      </c>
+      <c r="O93" t="inlineStr">
+        <is>
+          <t>Direct current revised local transport article source; verify whether current text is omitted or extant before route conclusions.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: add Stage 2C Bristol authority route control
</commit_message>
<xml_diff>
--- a/evidence/source_register.xlsx
+++ b/evidence/source_register.xlsx
@@ -7171,6 +7171,160 @@
         </is>
       </c>
     </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>SRC-LEG-0024</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>added-primary</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>1_must</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>statutory_and_business_case</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>UK legislation</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>Avon (Structural Change) Order 1995</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>1995</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>https://www.legislation.gov.uk/uksi/1995/493/made</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>evidence/raw/legislation/src-leg-0024_avon-structural-change-order-1995.html</t>
+        </is>
+      </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>downloaded</t>
+        </is>
+      </c>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>1_current_legislation</t>
+        </is>
+      </c>
+      <c r="M94" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="N94" t="inlineStr">
+        <is>
+          <t>41271ea2123e0e18240c90d62fc00e7be6526c605b31ed6300168377c4972010</t>
+        </is>
+      </c>
+      <c r="O94" t="inlineStr">
+        <is>
+          <t>Structural-change source for Bristol unitary and county-council status and transfer of county functions; supports competent-authority mapping when read with RTRA 1984 section 121A and Transport Act 2000 WPL provisions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>SRC-LEG-0025</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>added-primary</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>1_must</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>statutory_and_business_case</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>UK legislation</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>Transport Act 2000 section 163 road user charging schemes preliminary</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>https://www.legislation.gov.uk/ukpga/2000/38/section/163</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>evidence/raw/legislation/src-leg-0025_transport-act-2000-section-163-road-user-charging-schemes-preliminary.html</t>
+        </is>
+      </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>downloaded</t>
+        </is>
+      </c>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>1_current_legislation</t>
+        </is>
+      </c>
+      <c r="M95" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="N95" t="inlineStr">
+        <is>
+          <t>64c828cdc7da2cd6ea9e675ece757ec03d1e792f95be6c7000bd94800338211c</t>
+        </is>
+      </c>
+      <c r="O95" t="inlineStr">
+        <is>
+          <t>Direct cross-reference source for non-metropolitan local traffic authority construction used by Transport Act 2000 section 198.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: add Stage 2G WECA meeting search
</commit_message>
<xml_diff>
--- a/evidence/source_register.xlsx
+++ b/evidence/source_register.xlsx
@@ -7325,6 +7325,1007 @@
         </is>
       </c>
     </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>SRC-WECA-0017</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>added-primary</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>1_must</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>weca_governance</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>West of England Combined Authority ModernGov</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>Document search form</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>current_webpage</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>https://westofengland-ca.moderngov.co.uk/ieDocSearch.aspx?bcr=1</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>evidence/raw/west-of-england-mca/src-weca-0017_modern-gov-document-search-form.html</t>
+        </is>
+      </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>downloaded</t>
+        </is>
+      </c>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>3_formal_public_body_source</t>
+        </is>
+      </c>
+      <c r="M96" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="N96" t="inlineStr">
+        <is>
+          <t>2a09955b472472de2ce8a50bdf91411e45a06c282ec7201eb485aeff6fb65cec</t>
+        </is>
+      </c>
+      <c r="O96" t="inlineStr">
+        <is>
+          <t>Search form source for Stage 2G bounded official ModernGov meeting-record search.</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>SRC-WECA-0018</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>added-primary</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>1_must</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>weca_governance</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>West of England Combined Authority ModernGov</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>Joint MCA and Joint Committee meeting page 27 March 2026</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>https://westofengland-ca.moderngov.co.uk/ieListDocuments.aspx?CId=192&amp;MID=727</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>evidence/raw/west-of-england-mca/src-weca-0018_joint-mca-joint-committee-2026-03-27-meeting-page.html</t>
+        </is>
+      </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>downloaded</t>
+        </is>
+      </c>
+      <c r="L97" t="inlineStr">
+        <is>
+          <t>3_formal_public_body_source</t>
+        </is>
+      </c>
+      <c r="M97" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="N97" t="inlineStr">
+        <is>
+          <t>4eeacb3686b2ff7e3fb4d26f7ae9391bd5706622fa554305b5c8340fda361318</t>
+        </is>
+      </c>
+      <c r="O97" t="inlineStr">
+        <is>
+          <t>Meeting page reviewed for WPL workplace parking congestion charging CRSTS and mass transit hits.</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>SRC-WECA-0019</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>added-primary</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>1_must</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>weca_governance</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>West of England Combined Authority ModernGov</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>Joint MCA and Joint Committee meeting page 5 June 2026</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>https://westofengland-ca.moderngov.co.uk/ieListDocuments.aspx?CId=192&amp;MID=728</t>
+        </is>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>evidence/raw/west-of-england-mca/src-weca-0019_joint-mca-joint-committee-2026-06-05-meeting-page.html</t>
+        </is>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>downloaded</t>
+        </is>
+      </c>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t>3_formal_public_body_source</t>
+        </is>
+      </c>
+      <c r="M98" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="N98" t="inlineStr">
+        <is>
+          <t>63c095c073b576d5ea3ede41b890531ba643e6217858e4e86650abc9c90f0177</t>
+        </is>
+      </c>
+      <c r="O98" t="inlineStr">
+        <is>
+          <t>Meeting page reviewed for WPL workplace parking CAZ repayment CRSTS and funding-assurance hits.</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>SRC-WECA-0020</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>added-primary</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>1_must</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>weca_governance</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>West of England Combined Authority ModernGov</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>Overview and Scrutiny Committee meeting page 1 June 2026</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>https://westofengland-ca.moderngov.co.uk/ieListDocuments.aspx?CId=143&amp;MID=718</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>evidence/raw/west-of-england-mca/src-weca-0020_overview-scrutiny-2026-06-01-meeting-page.html</t>
+        </is>
+      </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>downloaded</t>
+        </is>
+      </c>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>3_formal_public_body_source</t>
+        </is>
+      </c>
+      <c r="M99" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="N99" t="inlineStr">
+        <is>
+          <t>cdada0a754f49f6a69864d13d6dbfd74a3e4aef5be309278f881dac9133bce8e</t>
+        </is>
+      </c>
+      <c r="O99" t="inlineStr">
+        <is>
+          <t>Overview and Scrutiny page reviewed for road user charging and congestion charging hits.</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>SRC-WECA-0021</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>added-primary</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>1_must</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>weca_governance</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>West of England Combined Authority ModernGov</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>Overview and Scrutiny Committee meeting page 23 March 2026</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>https://westofengland-ca.moderngov.co.uk/ieListDocuments.aspx?CId=143&amp;MID=716</t>
+        </is>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>evidence/raw/west-of-england-mca/src-weca-0021_overview-scrutiny-2026-03-23-meeting-page.html</t>
+        </is>
+      </c>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>downloaded</t>
+        </is>
+      </c>
+      <c r="L100" t="inlineStr">
+        <is>
+          <t>3_formal_public_body_source</t>
+        </is>
+      </c>
+      <c r="M100" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="N100" t="inlineStr">
+        <is>
+          <t>b12c214afe8cfd176b1b3108b28da4870ebf45accad1ea81c200e6241a7838f1</t>
+        </is>
+      </c>
+      <c r="O100" t="inlineStr">
+        <is>
+          <t>Overview and Scrutiny page reviewed for congestion charging and mass transit hits.</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>SRC-WECA-0022</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>added-primary</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>1_must</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>weca_governance</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>West of England Combined Authority ModernGov</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>Joint meeting 27 March 2026 public questions and Mayors responses</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>https://westofengland-ca.moderngov.co.uk/documents/s11483/Public%20Questions%20and%20Mayors%20Responses.pdf</t>
+        </is>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>evidence/raw/west-of-england-mca/src-weca-0022_joint-meeting-2026-03-27-public-questions-mayor-responses.pdf</t>
+        </is>
+      </c>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>downloaded</t>
+        </is>
+      </c>
+      <c r="L101" t="inlineStr">
+        <is>
+          <t>3_formal_public_body_source</t>
+        </is>
+      </c>
+      <c r="M101" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="N101" t="inlineStr">
+        <is>
+          <t>dfe663967731fc2f323960e44d43a3888f9ec966d977539e69f700580e202c0b</t>
+        </is>
+      </c>
+      <c r="O101" t="inlineStr">
+        <is>
+          <t>Public questions source produced transport and mass-transit hits but not formal Bristol WPL decision evidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>SRC-WECA-0023</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>added-primary</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>1_must</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>weca_governance</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>West of England Combined Authority ModernGov</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>Joint meeting 27 March 2026 statements</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>https://westofengland-ca.moderngov.co.uk/documents/s11484/Statements.pdf</t>
+        </is>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>evidence/raw/west-of-england-mca/src-weca-0023_joint-meeting-2026-03-27-statements.pdf</t>
+        </is>
+      </c>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>downloaded</t>
+        </is>
+      </c>
+      <c r="L102" t="inlineStr">
+        <is>
+          <t>3_formal_public_body_source</t>
+        </is>
+      </c>
+      <c r="M102" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="N102" t="inlineStr">
+        <is>
+          <t>8e8a2c92299b03311b3c95b87dd75042dbe7669e4e0e5a32c91cf9b94b405c99</t>
+        </is>
+      </c>
+      <c r="O102" t="inlineStr">
+        <is>
+          <t>Public statements source produced false-positive workplace parking levy search hits and no formal Bristol WPL decision evidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>SRC-WECA-0024</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>added-primary</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>1_must</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>weca_assurance</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>West of England Combined Authority ModernGov</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>Joint meeting 27 March 2026 transport report</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>https://westofengland-ca.moderngov.co.uk/documents/s11253/Item%2013%20-%20Transport.pdf</t>
+        </is>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>evidence/raw/west-of-england-mca/src-weca-0024_joint-meeting-2026-03-27-transport-report.pdf</t>
+        </is>
+      </c>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>downloaded</t>
+        </is>
+      </c>
+      <c r="L103" t="inlineStr">
+        <is>
+          <t>3_formal_public_body_source</t>
+        </is>
+      </c>
+      <c r="M103" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="N103" t="inlineStr">
+        <is>
+          <t>83f486882c76c2cfc56c88149333608ad618221ec6564293ac1fac59aa66e082</t>
+        </is>
+      </c>
+      <c r="O103" t="inlineStr">
+        <is>
+          <t>Transport report source for CRSTS mass transit and funding-assurance interface context only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>SRC-WECA-0025</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>added-primary</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>1_must</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>weca_governance</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>West of England Combined Authority ModernGov</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>Joint meeting 5 June 2026 public questions and Mayors responses</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>https://westofengland-ca.moderngov.co.uk/documents/s11641/FINAL%20-%20Public%20Questions%20and%20Mayors%20Responses.pdf</t>
+        </is>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>evidence/raw/west-of-england-mca/src-weca-0025_joint-meeting-2026-06-05-public-questions-mayor-responses.pdf</t>
+        </is>
+      </c>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>downloaded</t>
+        </is>
+      </c>
+      <c r="L104" t="inlineStr">
+        <is>
+          <t>3_formal_public_body_source</t>
+        </is>
+      </c>
+      <c r="M104" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="N104" t="inlineStr">
+        <is>
+          <t>895019e3bd6eeb1c1107babb40d0688fb580f8cfe0b48d1664bc37f90a266514</t>
+        </is>
+      </c>
+      <c r="O104" t="inlineStr">
+        <is>
+          <t>Public questions source reviewed for workplace parking road user charging and transport hits; no formal Bristol WPL decision evidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>SRC-WECA-0026</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>added-primary</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>1_must</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>weca_governance</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>West of England Combined Authority ModernGov</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>Joint meeting 5 June 2026 statements</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>https://westofengland-ca.moderngov.co.uk/documents/s11626/FINAL%20-%20Statements%20to%20WECA%20WEJC.pdf</t>
+        </is>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>evidence/raw/west-of-england-mca/src-weca-0026_joint-meeting-2026-06-05-statements.pdf</t>
+        </is>
+      </c>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>downloaded</t>
+        </is>
+      </c>
+      <c r="L105" t="inlineStr">
+        <is>
+          <t>3_formal_public_body_source</t>
+        </is>
+      </c>
+      <c r="M105" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="N105" t="inlineStr">
+        <is>
+          <t>dca40b317372ae37a54bc87c8afc592004331c742d08e143616f5753fd049990</t>
+        </is>
+      </c>
+      <c r="O105" t="inlineStr">
+        <is>
+          <t>Public statements source reviewed for WPL-adjacent token hits; no formal Bristol WPL decision evidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>SRC-WECA-0027</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>added-primary</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>1_must</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>weca_assurance</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>West of England Combined Authority ModernGov</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>Joint meeting 5 June 2026 MCA and mayoral budget outturn</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>https://westofengland-ca.moderngov.co.uk/documents/s11517/Item%2008%20-%20MCA%20Mayoral%20Budget%20Outturn.pdf</t>
+        </is>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>evidence/raw/west-of-england-mca/src-weca-0027_joint-meeting-2026-06-05-mca-mayoral-budget-outturn.pdf</t>
+        </is>
+      </c>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>downloaded</t>
+        </is>
+      </c>
+      <c r="L106" t="inlineStr">
+        <is>
+          <t>3_formal_public_body_source</t>
+        </is>
+      </c>
+      <c r="M106" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="N106" t="inlineStr">
+        <is>
+          <t>c9bc2c082114b7f8edc236fae2ab46a5ba83c1b5e293c58b4880f6105954a294</t>
+        </is>
+      </c>
+      <c r="O106" t="inlineStr">
+        <is>
+          <t>Budget outturn source produced token-match WPL hits and CAZ CRSTS transport context but no Bristol WPL funding decision evidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>SRC-WECA-0028</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>added-primary</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>1_must</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>weca_assurance</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>West of England Combined Authority ModernGov</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>Joint meeting 5 June 2026 Investment Fund Programme and Grant Assurance</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>https://westofengland-ca.moderngov.co.uk/documents/s11539/Item%2009%20-%20Investment%20Fund%20Programme.pdf</t>
+        </is>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>evidence/raw/west-of-england-mca/src-weca-0028_joint-meeting-2026-06-05-investment-fund-programme.pdf</t>
+        </is>
+      </c>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>downloaded</t>
+        </is>
+      </c>
+      <c r="L107" t="inlineStr">
+        <is>
+          <t>3_formal_public_body_source</t>
+        </is>
+      </c>
+      <c r="M107" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="N107" t="inlineStr">
+        <is>
+          <t>6b5869048c5c46ac09485abea69b24b9dd9134c5e76b2e21afb15abf8df1a06b</t>
+        </is>
+      </c>
+      <c r="O107" t="inlineStr">
+        <is>
+          <t>Investment and grant assurance source reviewed for transport levy parking investment and Bristol package context; no Bristol WPL approval evidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>SRC-WECA-0029</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>added-primary</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>1_must</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>weca_assurance</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>West of England Combined Authority ModernGov</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>Joint meeting 5 June 2026 Delivery Assurance</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>https://westofengland-ca.moderngov.co.uk/documents/s11519/Item%2010%20-%20Delivery%20Assurance.pdf</t>
+        </is>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>evidence/raw/west-of-england-mca/src-weca-0029_joint-meeting-2026-06-05-delivery-assurance.pdf</t>
+        </is>
+      </c>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>downloaded</t>
+        </is>
+      </c>
+      <c r="L108" t="inlineStr">
+        <is>
+          <t>3_formal_public_body_source</t>
+        </is>
+      </c>
+      <c r="M108" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="N108" t="inlineStr">
+        <is>
+          <t>b4bb965add8d256e58c1de657184ac3dd608f7e1387ee437f1a45e4243c4ff13</t>
+        </is>
+      </c>
+      <c r="O108" t="inlineStr">
+        <is>
+          <t>Delivery assurance source for CRSTS risk-budget and programme assurance context only.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: add Stage 2J DfT process controls
</commit_message>
<xml_diff>
--- a/evidence/source_register.xlsx
+++ b/evidence/source_register.xlsx
@@ -8326,6 +8326,160 @@
         </is>
       </c>
     </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>SRC-DFT-0003</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>added-primary</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>1_must</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>statutory_and_business_case</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>GOV.UK Search</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>GOV.UK bounded search - workplace parking levy confirmation Secretary of State</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>https://www.gov.uk/search/all?keywords=workplace%20parking%20levy%20confirmation%20Secretary%20of%20State&amp;order=relevance</t>
+        </is>
+      </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>evidence/raw/dft-and-tag/src-dft-0003_govuk-search-wpl-confirmation-sos.html</t>
+        </is>
+      </c>
+      <c r="K109" t="inlineStr">
+        <is>
+          <t>downloaded</t>
+        </is>
+      </c>
+      <c r="L109" t="inlineStr">
+        <is>
+          <t>2_official_government_guidance</t>
+        </is>
+      </c>
+      <c r="M109" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="N109" t="inlineStr">
+        <is>
+          <t>58b440d0cc118e10574e5dba3d9da5fc987fcf84a4907a38ca115e5e923dd9ec</t>
+        </is>
+      </c>
+      <c r="O109" t="inlineStr">
+        <is>
+          <t>Search-control source for Stage 2J; not substantive procedural guidance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>SRC-DFT-0004</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>added-primary</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>1_must</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>statutory_and_business_case</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>GOV.UK Search</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>GOV.UK bounded search - workplace parking levy DfT</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>https://www.gov.uk/search/all?keywords=workplace%20parking%20levy%20DfT&amp;order=relevance</t>
+        </is>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>evidence/raw/dft-and-tag/src-dft-0004_src-dft-0004-govuk-search-workplace-parking-levy-dft.html</t>
+        </is>
+      </c>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>downloaded</t>
+        </is>
+      </c>
+      <c r="L110" t="inlineStr">
+        <is>
+          <t>2_official_government_guidance</t>
+        </is>
+      </c>
+      <c r="M110" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="N110" t="inlineStr">
+        <is>
+          <t>618c441b8be53659490818595418e1a2498c48e0eccd1e0d11769278a6a30501</t>
+        </is>
+      </c>
+      <c r="O110" t="inlineStr">
+        <is>
+          <t>Search-control source for Stage 2J; not substantive procedural guidance.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: add Stage 2K order change controls
</commit_message>
<xml_diff>
--- a/evidence/source_register.xlsx
+++ b/evidence/source_register.xlsx
@@ -8480,6 +8480,160 @@
         </is>
       </c>
     </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>SRC-LEG-0026</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>added-primary</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>1_must</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>statutory_and_business_case</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>UK legislation</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>Transport Act 2000 section 183 licensing schemes to be made by order</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>https://www.legislation.gov.uk/ukpga/2000/38/section/183</t>
+        </is>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>evidence/raw/legislation/src-leg-0026_src-leg-0026-transport-act-2000-section-183-licensing-schemes-order.html</t>
+        </is>
+      </c>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>downloaded</t>
+        </is>
+      </c>
+      <c r="L111" t="inlineStr">
+        <is>
+          <t>1_current_legislation</t>
+        </is>
+      </c>
+      <c r="M111" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="N111" t="inlineStr">
+        <is>
+          <t>2316db5bca741770fe06d31e4133badb473d7428769117c69cfcab2b0a039018</t>
+        </is>
+      </c>
+      <c r="O111" t="inlineStr">
+        <is>
+          <t>Direct current-law source for making variation and revocation of WPL licensing schemes by order.</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>SRC-LEG-0027</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>added-primary</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>1_must</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>statutory_and_business_case</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>UK legislation</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>Transport Act 2000 section 185 licensing schemes consultation and inquiries</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>https://www.legislation.gov.uk/ukpga/2000/38/section/185</t>
+        </is>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>evidence/raw/legislation/src-leg-0027_src-leg-0027-transport-act-2000-section-185-consultation-inquiries.html</t>
+        </is>
+      </c>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>downloaded</t>
+        </is>
+      </c>
+      <c r="L112" t="inlineStr">
+        <is>
+          <t>1_current_legislation</t>
+        </is>
+      </c>
+      <c r="M112" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="N112" t="inlineStr">
+        <is>
+          <t>e8d4e65fe4f1a56883d2c8ff11d1e35069a4baf445107f5ca411cc484bcd4e29</t>
+        </is>
+      </c>
+      <c r="O112" t="inlineStr">
+        <is>
+          <t>Direct current-law source for WPL consultation and inquiry controls.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: add Stage 14B secret scan controls
</commit_message>
<xml_diff>
--- a/evidence/source_register.xlsx
+++ b/evidence/source_register.xlsx
@@ -448,7 +448,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>downloaded</t>
+          <t>downloaded_raw_omitted_from_public_repo</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -468,7 +468,7 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Large file; useful for ensuring no appendix is missed.</t>
+          <t>Large file; useful for ensuring no appendix is missed. Raw public PDF omitted from GitHub after GitGuardian legacy Grafana/Power BI token-pattern collision; retain source URL and hash, reacquire outside the public repo if raw binary inspection is needed.</t>
         </is>
       </c>
     </row>
@@ -987,7 +987,7 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>downloaded</t>
+          <t>downloaded_raw_omitted_from_public_repo</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -1007,7 +1007,7 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Use for triangulating public and councillor challenges.</t>
+          <t>Use for triangulating public and councillor challenges. Raw public PDF omitted from GitHub after GitGuardian legacy Grafana/Power BI token-pattern collision; retain source URL and hash, reacquire outside the public repo if raw binary inspection is needed.</t>
         </is>
       </c>
     </row>
@@ -1295,7 +1295,7 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>downloaded</t>
+          <t>downloaded_raw_omitted_from_public_repo</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
@@ -1315,7 +1315,7 @@
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>Large file; useful for capturing public forum and forward-looking timetable.</t>
+          <t>Large file; useful for capturing public forum and forward-looking timetable. Raw public PDF omitted from GitHub after GitGuardian legacy Grafana/Power BI token-pattern collision; retain source URL and hash, reacquire outside the public repo if raw binary inspection is needed.</t>
         </is>
       </c>
     </row>

</xml_diff>